<commit_message>
resync to current version
</commit_message>
<xml_diff>
--- a/migrations/solutions-migration-coverage.xlsx
+++ b/migrations/solutions-migration-coverage.xlsx
@@ -8536,25 +8536,25 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>benefits_-_*  (media collage)</t>
+          <t>benefits_-_*  (media collage) — DISABLED, see notes</t>
         </is>
       </c>
       <c r="B6" s="14" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (was 17/87, now 0)</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>heading + paragraph + main image + 2 floating circle images (content-collage pattern)</t>
+          <t>(none — script now always returns empty for children)</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Matches the "Make your mission a movement" collage already built on the rebuilt Fundraising hub page.</t>
+          <t>CORRECTED 2026-07-21: benefits_-_enable_benefits_media_section is true on 17 legacy children, but the section does not appear on any of their live legacy pages (checked 2, different families, both show the accordion Benefits/Approach section instead). benefits_-_title/description/floating_image_1/2 are byte-identical across all 17 posts — stale template boilerplate, not real per-post content. Appears to be a hub-page-only design element. momentive_sol_benefits_media_block() now unconditionally returns '' for children; see its docblock in migrate-solutions.php.</t>
         </is>
       </c>
     </row>

</xml_diff>